<commit_message>
updates quotes integrating new feedback, cleans up code
</commit_message>
<xml_diff>
--- a/feedback/quantitative_themes.xlsx
+++ b/feedback/quantitative_themes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\data-dock\feedback\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F420A0AB-71E6-4780-B1F9-BC7AF5063382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F982E686-97E7-499E-B44D-3C97400B8FCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -340,6 +340,17 @@
     <t>Controls/Filters</t>
   </si>
   <si>
+    <t>“Year slider… difficult to use rather than choosing a date range.”
+“Could use summary data type (month, year) for box plots.”
+“Year toggle label should be ‘Water Year’.”
+“Tick marks in the year toggle were confusing.”
+“Would like to go more specific than one year.”
+“Options appearing/disappearing when selecting sites/analytes.”
+"I tried searching just by copying the sites into the search. P8 didn't come up in the search bar as written. Had to write P08. Again, easy to fix, just annoying." 
+"I'm not sure if I like the auto-zoom/pan; when I want to select multiple points on the map I have to zoom back out every time." 
+"The only way to see which stations are inactive is by the dot color on the map but once you select it you can't tell anymore."</t>
+  </si>
+  <si>
     <t>Visualization/Data</t>
   </si>
   <si>
@@ -350,7 +361,8 @@
 “Add stations upstream of Sacramento at Hood.”
 “Compare field length assignments to genetic results.”
 “Connections to EDI pages / metadata / downloads.”
-“Box plots across time instead of one big box plot.”</t>
+“Box plots across time instead of one big box plot.”
+"Water quality tab doesn't show cities so it was a little confusing to orient myself not being familiar with the delta."</t>
   </si>
   <si>
     <t>"Need a ‘no data’ message when inactive site selected.”
@@ -363,14 +375,6 @@
 “Going between sites and analytes got pretty confusing. Options would appear/disappear.”
 “Seems good for finding something specific but difficult to explore openly.”
 “Inactive site selection was confusing.”</t>
-  </si>
-  <si>
-    <t xml:space="preserve">“Year slider… difficult to use rather than choosing a date range.”
-“Could use summary data type (month, year) for box plots.”
-“Year toggle label should be ‘Water Year’.”
-“Tick marks in the year toggle were confusing.”
-“Would like to go more specific than one year.”
-“Options appearing/disappearing when selecting sites/analytes.” </t>
   </si>
 </sst>
 </file>
@@ -609,15 +613,13 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1061,8 +1063,8 @@
       <c r="A17" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>31</v>
+      <c r="B17" s="15" t="s">
+        <v>32</v>
       </c>
       <c r="C17" s="12"/>
     </row>
@@ -1071,16 +1073,16 @@
         <v>27</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C18" s="12"/>
     </row>
     <row r="19" spans="1:3" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B19" s="13" t="s">
         <v>29</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>30</v>
       </c>
       <c r="C19" s="12"/>
     </row>
@@ -1088,10 +1090,10 @@
       <c r="A20" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C20" s="15"/>
+      <c r="B20" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>